<commit_message>
Add role based admin dashboards and routing
</commit_message>
<xml_diff>
--- a/exports/crewholic_database.xlsx
+++ b/exports/crewholic_database.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="35">
   <si>
     <t>_id</t>
   </si>
@@ -28,6 +28,9 @@
     <t>password</t>
   </si>
   <si>
+    <t>authProvider</t>
+  </si>
+  <si>
     <t>role</t>
   </si>
   <si>
@@ -40,25 +43,25 @@
     <t>__v</t>
   </si>
   <si>
-    <t>authProvider</t>
-  </si>
-  <si>
-    <t>"6a03ec2f18d4cbb64a06b37a"</t>
-  </si>
-  <si>
-    <t>RONIT MISHRA</t>
-  </si>
-  <si>
-    <t>ronitmishra5555@gmail.com</t>
-  </si>
-  <si>
-    <t>$2b$10$AH7gkM0gyU0a0aMC4Sgfe.tObPHOD1hQsZMHFP5kvpF1IpFuWgavq</t>
-  </si>
-  <si>
-    <t>super_admin</t>
-  </si>
-  <si>
-    <t>"6a040f90b284dd0238e19dac"</t>
+    <t>"6a1d180acb20cec17da27ae6"</t>
+  </si>
+  <si>
+    <t>Sumit Kumar Rout</t>
+  </si>
+  <si>
+    <t>srout2023@gift.edu.in</t>
+  </si>
+  <si>
+    <t>$2b$10$4qVSycuvB1wbiVZLR4t.sexbx0s9iI2DulwdeMwS03yUmBr.NBYz6</t>
+  </si>
+  <si>
+    <t>local</t>
+  </si>
+  <si>
+    <t>finance_admin</t>
+  </si>
+  <si>
+    <t>"6a1d18d3e63ebf0b0301f426"</t>
   </si>
   <si>
     <t>Main Admin</t>
@@ -67,111 +70,27 @@
     <t>admin@crewholic.com</t>
   </si>
   <si>
-    <t>$2b$10$kJbRlqANMqA3pvAlRzQDze1fvYJ5ylBikklbYHqJmX/M46Bbkfc46</t>
-  </si>
-  <si>
-    <t>"6a0447b2453fcba87821e4e8"</t>
-  </si>
-  <si>
-    <t>SUMIT ROUT</t>
-  </si>
-  <si>
-    <t>srout2023@gift.edu.in</t>
-  </si>
-  <si>
-    <t>$2b$10$O7grwdYVQ/dKmp4.U4AvXOWahskXN/03c5irSRY110GXk.aTr25s2</t>
+    <t>$2b$10$aCQM3domoCTfgDqrja6qseO0fF5iFWGeR9ugTP58/.ZiB2l9W4KmK</t>
+  </si>
+  <si>
+    <t>admin</t>
+  </si>
+  <si>
+    <t>"6a1d1affbbd58b1c59a425fc"</t>
+  </si>
+  <si>
+    <t>Mamata Rout</t>
+  </si>
+  <si>
+    <t>sumitkmrrt@gmail.com</t>
+  </si>
+  <si>
+    <t>$2b$10$47AYdm5Yey9dTavPsm.X5eOhtxts306sSQEZvlUOQXkjkVpX4y0jy</t>
   </si>
   <si>
     <t>user</t>
   </si>
   <si>
-    <t>"6a04482b453fcba87821e4e9"</t>
-  </si>
-  <si>
-    <t>Mamata ROUT</t>
-  </si>
-  <si>
-    <t>smsteam@gift.edu.in</t>
-  </si>
-  <si>
-    <t>$2b$10$/fJ1pWbcPKHyv.YFUsdXZ.Hjux3Ch2avYY/PiNmCkxuOZ0/Noq4jS</t>
-  </si>
-  <si>
-    <t>"6a14338402b3c40cdd25a0b6"</t>
-  </si>
-  <si>
-    <t>Sumit Kumar Rout</t>
-  </si>
-  <si>
-    <t>srout2023@gmail.com</t>
-  </si>
-  <si>
-    <t>$2b$10$rVvZZUPVXBNlSsRe5xfDReDgFMHbIJUIXOLyUU43UX0BKfBKfoDM2</t>
-  </si>
-  <si>
-    <t>local</t>
-  </si>
-  <si>
-    <t>"6a1438f138843a42469ef775"</t>
-  </si>
-  <si>
-    <t>Sutarrdeba</t>
-  </si>
-  <si>
-    <t>srout2000@gmail.com</t>
-  </si>
-  <si>
-    <t>$2b$10$yiWogQrdiTwVZVjXO.1.GOCWrwtQvNdFHl0Hf5JNCnBOynH92JMgG</t>
-  </si>
-  <si>
-    <t>"6a1568bc5208d43e32c98351"</t>
-  </si>
-  <si>
-    <t>SUMIT Jena</t>
-  </si>
-  <si>
-    <t>srout2008@gmail.com</t>
-  </si>
-  <si>
-    <t>$2b$10$ePJb.uAdNY8h6r13.wVuiO38mVtcAxa8zy/ZIad1oOjRwZbHwvSOK</t>
-  </si>
-  <si>
-    <t>"6a1569cf5208d43e32c98352"</t>
-  </si>
-  <si>
-    <t>Mamata  Jena</t>
-  </si>
-  <si>
-    <t>srout2015@gmail.com</t>
-  </si>
-  <si>
-    <t>$2b$10$n3TvZ60IFifff7muICuH4uGdHsqfkq7rdg3Ic2i6R.lUnEt5aXg/.</t>
-  </si>
-  <si>
-    <t>"6a156b8b5208d43e32c98353"</t>
-  </si>
-  <si>
-    <t>Ronit Das</t>
-  </si>
-  <si>
-    <t>srout2010@gmail.com</t>
-  </si>
-  <si>
-    <t>$2b$10$DKJP20Xr6tw5aAy4Erx7Aea6e4BrqDBVwnWNBrRa9SJZksUbOMdSy</t>
-  </si>
-  <si>
-    <t>"6a19bfb3c06de434728623f0"</t>
-  </si>
-  <si>
-    <t>Suprabha Subhadarshini Rout</t>
-  </si>
-  <si>
-    <t>sumitkmrrt@gmail.com</t>
-  </si>
-  <si>
-    <t>$2b$10$fwr.Y1jE3TSH5SIczNo/v.71GR2OGMJ0DDPu8XcttFqT01kmxYOpy</t>
-  </si>
-  <si>
     <t>service</t>
   </si>
   <si>
@@ -200,9 +119,6 @@
   </si>
   <si>
     <t>$2b$10$2yBifcmgd6Tp/1FhNJyAQ.nMRrunmtCCK7hR.Y/NFvT3R/PTjVXZi</t>
-  </si>
-  <si>
-    <t>admin</t>
   </si>
 </sst>
 </file>
@@ -580,7 +496,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="9" width="25" customWidth="1"/>
@@ -615,7 +531,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -631,266 +547,75 @@
       <c r="E2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="1">
-        <v>46155.13388141204</v>
+      <c r="F2" t="s">
+        <v>14</v>
       </c>
       <c r="G2" s="1">
-        <v>46155.13388141204</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>46174.22679075232</v>
+      </c>
+      <c r="H2" s="1">
+        <v>46174.22679075232</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E3" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="1">
-        <v>46155.238708171295</v>
+      <c r="F3" t="s">
+        <v>19</v>
       </c>
       <c r="G3" s="1">
-        <v>46155.238708171295</v>
-      </c>
-      <c r="H3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+        <v>46174.229111469904</v>
+      </c>
+      <c r="H3" s="1">
+        <v>46174.229111469904</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" s="1">
-        <v>46155.40503268519</v>
+        <v>13</v>
+      </c>
+      <c r="F4" t="s">
+        <v>24</v>
       </c>
       <c r="G4" s="1">
-        <v>46155.40503268519</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="1">
-        <v>46155.406425231486</v>
-      </c>
-      <c r="G5" s="1">
-        <v>46155.406425231486</v>
-      </c>
-      <c r="H5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" t="s">
-        <v>30</v>
-      </c>
-      <c r="E6" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" s="1">
-        <v>46167.48153798611</v>
-      </c>
-      <c r="G6" s="1">
-        <v>46167.48153798611</v>
-      </c>
-      <c r="H6">
-        <v>0</v>
-      </c>
-      <c r="I6" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B7" t="s">
-        <v>33</v>
-      </c>
-      <c r="C7" t="s">
-        <v>34</v>
-      </c>
-      <c r="D7" t="s">
-        <v>35</v>
-      </c>
-      <c r="E7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F7" s="1">
-        <v>46167.49760673611</v>
-      </c>
-      <c r="G7" s="1">
-        <v>46167.49760673611</v>
-      </c>
-      <c r="H7">
-        <v>0</v>
-      </c>
-      <c r="I7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" t="s">
-        <v>38</v>
-      </c>
-      <c r="D8" t="s">
-        <v>39</v>
-      </c>
-      <c r="E8" t="s">
-        <v>22</v>
-      </c>
-      <c r="F8" s="1">
-        <v>46168.39773858796</v>
-      </c>
-      <c r="G8" s="1">
-        <v>46168.39773858796</v>
-      </c>
-      <c r="H8">
-        <v>0</v>
-      </c>
-      <c r="I8" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>40</v>
-      </c>
-      <c r="B9" t="s">
-        <v>41</v>
-      </c>
-      <c r="C9" t="s">
-        <v>42</v>
-      </c>
-      <c r="D9" t="s">
-        <v>43</v>
-      </c>
-      <c r="E9" t="s">
-        <v>22</v>
-      </c>
-      <c r="F9" s="1">
-        <v>46168.40092369213</v>
-      </c>
-      <c r="G9" s="1">
-        <v>46168.40092369213</v>
-      </c>
-      <c r="H9">
-        <v>0</v>
-      </c>
-      <c r="I9" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>44</v>
-      </c>
-      <c r="B10" t="s">
-        <v>45</v>
-      </c>
-      <c r="C10" t="s">
-        <v>46</v>
-      </c>
-      <c r="D10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E10" t="s">
-        <v>22</v>
-      </c>
-      <c r="F10" s="1">
-        <v>46168.40605329861</v>
-      </c>
-      <c r="G10" s="1">
-        <v>46168.40605329861</v>
-      </c>
-      <c r="H10">
-        <v>0</v>
-      </c>
-      <c r="I10" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>48</v>
-      </c>
-      <c r="B11" t="s">
-        <v>49</v>
-      </c>
-      <c r="C11" t="s">
-        <v>50</v>
-      </c>
-      <c r="D11" t="s">
-        <v>51</v>
-      </c>
-      <c r="E11" t="s">
-        <v>22</v>
-      </c>
-      <c r="F11" s="1">
-        <v>46171.68948450232</v>
-      </c>
-      <c r="G11" s="1">
-        <v>46171.68948450232</v>
-      </c>
-      <c r="H11">
-        <v>0</v>
-      </c>
-      <c r="I11" t="s">
-        <v>31</v>
+        <v>46174.23554511574</v>
+      </c>
+      <c r="H4" s="1">
+        <v>46174.23554511574</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -912,36 +637,36 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="C1" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="D1" t="s">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="E1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="C2">
         <v>2000</v>
       </c>
       <c r="D2" t="s">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="E2" s="1">
         <v>46145.68469171296</v>
@@ -955,16 +680,16 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="B3" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="C3">
         <v>2000</v>
       </c>
       <c r="D3" t="s">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="E3" s="1">
         <v>46145.69621173611</v>
@@ -1004,30 +729,30 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>60</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>61</v>
+        <v>34</v>
       </c>
       <c r="E2" t="s">
-        <v>62</v>
+        <v>19</v>
       </c>
       <c r="F2" s="1">
         <v>46141.26088069445</v>

</xml_diff>

<commit_message>
Fix production API base URL and auth flow
</commit_message>
<xml_diff>
--- a/exports/crewholic_database.xlsx
+++ b/exports/crewholic_database.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="33">
   <si>
     <t>_id</t>
   </si>
@@ -43,6 +43,9 @@
     <t>__v</t>
   </si>
   <si>
+    <t>isActive</t>
+  </si>
+  <si>
     <t>"6a1d180acb20cec17da27ae6"</t>
   </si>
   <si>
@@ -58,7 +61,7 @@
     <t>local</t>
   </si>
   <si>
-    <t>finance_admin</t>
+    <t>rental_admin</t>
   </si>
   <si>
     <t>"6a1d18d3e63ebf0b0301f426"</t>
@@ -91,25 +94,16 @@
     <t>user</t>
   </si>
   <si>
-    <t>service</t>
-  </si>
-  <si>
-    <t>amount</t>
-  </si>
-  <si>
-    <t>status</t>
-  </si>
-  <si>
-    <t>"69f777156176d65c3d1e8f16"</t>
-  </si>
-  <si>
-    <t>rental</t>
-  </si>
-  <si>
-    <t>pending</t>
-  </si>
-  <si>
-    <t>"69f77af8416476c6f630c038"</t>
+    <t>"6a258130f689f245c896c297"</t>
+  </si>
+  <si>
+    <t>Ronit Kumar Mishra</t>
+  </si>
+  <si>
+    <t>ronitmishra5555@gmail.com</t>
+  </si>
+  <si>
+    <t>$2b$10$m3QZCcj2fIYN0qJuAAXxqe9iBh4gJLieR5FJPeFua4zYxANBXbWHq</t>
   </si>
   <si>
     <t>"69f1a20c74b2a9b4a0eff7bc"</t>
@@ -496,13 +490,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="9" width="25" customWidth="1"/>
+    <col min="1" max="10" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -529,26 +523,29 @@
       </c>
       <c r="I1" t="s">
         <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G2" s="1">
         <v>46174.22679075232</v>
@@ -562,22 +559,22 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G3" s="1">
         <v>46174.229111469904</v>
@@ -591,22 +588,22 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G4" s="1">
         <v>46174.23554511574</v>
@@ -616,6 +613,38 @@
       </c>
       <c r="I4">
         <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="1">
+        <v>46180.606488854166</v>
+      </c>
+      <c r="H5" s="1">
+        <v>46180.606488854166</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -626,82 +655,9 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="7" width="25" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C2">
-        <v>2000</v>
-      </c>
-      <c r="D2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E2" s="1">
-        <v>46145.68469171296</v>
-      </c>
-      <c r="F2" s="1">
-        <v>46145.68469171296</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C3">
-        <v>2000</v>
-      </c>
-      <c r="D3" t="s">
-        <v>30</v>
-      </c>
-      <c r="E3" s="1">
-        <v>46145.69621173611</v>
-      </c>
-      <c r="F3" s="1">
-        <v>46145.69621173611</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -740,19 +696,19 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
         <v>32</v>
       </c>
-      <c r="B2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D2" t="s">
-        <v>34</v>
-      </c>
       <c r="E2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F2" s="1">
         <v>46141.26088069445</v>

</xml_diff>